<commit_message>
feat: recover 2026-05-19 GTC class + attendance for May 12/19/26
- Restore 2026-05-19 from backup. The audio was mislabeled (several
  recordings mixed), not a private call: it contained a real GTC class
  plus unrelated content. Trimmed to GTC-only blocks; removed Spanish,
  an unrelated biology lesson, productivity coaching and a private phone
  call. Result: English-only, 0% Spanish, no private content.
- Mark all 5 students present for May 12, 19 and 26 (attendance table +
  calendar status).
- Fix process_class.py --skip-transcription so it rebuilds from an
  existing transcript_cache without needing audio_blocks info.
</commit_message>
<xml_diff>
--- a/docs/Component_A_Aggregated.xlsx
+++ b/docs/Component_A_Aggregated.xlsx
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-31 12:36 · 8 classes</t>
+          <t>Generated: 2026-06-01 12:44 · 9 classes</t>
         </is>
       </c>
     </row>
@@ -594,105 +594,105 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2.97</v>
+        <v>2.94</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="6" t="n">
-        <v>3.71</v>
+        <v>3.65</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>11.68</v>
+        <v>11.59</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>58.4</v>
+        <v>58</v>
       </c>
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="6" t="n">
-        <v>5.21</v>
+        <v>5.15</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>13.18</v>
+        <v>13.09</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>65.90000000000001</v>
+        <v>65.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Chilaka</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>2.44</v>
+        <v>2.97</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="6" t="n">
-        <v>3.92</v>
+        <v>3.41</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>11.35</v>
+        <v>11.39</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>56.8</v>
+        <v>57</v>
       </c>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="6" t="n">
-        <v>5.17</v>
+        <v>4.08</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>12.6</v>
+        <v>12.06</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>63</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Chilaka</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2.41</v>
+        <v>2.44</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
       <c r="F7" s="6" t="n">
-        <v>3.37</v>
+        <v>3.86</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.78</v>
+        <v>11.31</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>53.9</v>
+        <v>56.5</v>
       </c>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="6" t="n">
-        <v>4.06</v>
+        <v>5.14</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>11.47</v>
+        <v>12.58</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>57.4</v>
+        <v>62.9</v>
       </c>
     </row>
     <row r="8">
@@ -702,33 +702,33 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2.57</v>
+        <v>2.93</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="6" t="n">
-        <v>3.18</v>
+        <v>3.19</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>10.75</v>
+        <v>11.12</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>53.8</v>
+        <v>55.6</v>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="6" t="n">
-        <v>4.06</v>
+        <v>4.02</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>11.63</v>
+        <v>11.95</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>58.1</v>
+        <v>59.7</v>
       </c>
     </row>
     <row r="9">
@@ -738,17 +738,17 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2.37</v>
+        <v>2.32</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="6" t="n">
-        <v>3.25</v>
+        <v>3.31</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>10.63</v>
@@ -758,13 +758,13 @@
       </c>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="6" t="n">
-        <v>4.57</v>
+        <v>4.59</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>11.94</v>
+        <v>11.91</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>59.7</v>
+        <v>59.6</v>
       </c>
     </row>
   </sheetData>
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -791,6 +791,7 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -843,10 +844,15 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="J3" s="12" t="inlineStr">
+      <c r="K3" s="12" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
@@ -880,78 +886,87 @@
         <v>11.9</v>
       </c>
       <c r="I4" s="6" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="J4" s="6" t="n">
         <v>11.53</v>
       </c>
-      <c r="J4" s="7" t="n">
-        <v>11.68</v>
+      <c r="K4" s="7" t="n">
+        <v>11.59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Chilaka</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>11</v>
+        <v>8.33</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>12.59</v>
+        <v>13.23</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>10</v>
+        <v>11.37</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>11.54</v>
+        <v>11.73</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>9.220000000000001</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>11.02</v>
+        <v>9.16</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>12.41</v>
+        <v>12.46</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13.05</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>11.35</v>
+        <v>16.25</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>10.42</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>11.39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Chilaka</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>8.33</v>
+        <v>11</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>13.23</v>
+        <v>12.59</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>11.37</v>
+        <v>10</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>11.73</v>
+        <v>11.54</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>9.550000000000001</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>9.16</v>
+        <v>11.02</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>12.46</v>
+        <v>12.41</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.42</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>10.78</v>
+        <v>10.93</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>11.31</v>
       </c>
     </row>
     <row r="7">
@@ -982,10 +997,13 @@
         <v>12.43</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="J7" s="6" t="n">
         <v>11.07</v>
       </c>
-      <c r="J7" s="7" t="n">
-        <v>10.75</v>
+      <c r="K7" s="7" t="n">
+        <v>11.12</v>
       </c>
     </row>
     <row r="8">
@@ -1016,9 +1034,12 @@
         <v>12.08</v>
       </c>
       <c r="I8" s="6" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="J8" s="6" t="n">
         <v>12.67</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="K8" s="7" t="n">
         <v>10.63</v>
       </c>
     </row>
@@ -1033,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1046,6 +1067,7 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1098,10 +1120,15 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
@@ -1135,78 +1162,87 @@
         <v>13.4</v>
       </c>
       <c r="I4" s="6" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="J4" s="6" t="n">
         <v>13.03</v>
       </c>
-      <c r="J4" s="9" t="n">
-        <v>13.18</v>
+      <c r="K4" s="9" t="n">
+        <v>13.09</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Chilaka</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>12.5</v>
+        <v>8.33</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>13.59</v>
+        <v>13.73</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>10</v>
+        <v>12.37</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>13.04</v>
+        <v>12.73</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>10.72</v>
+        <v>10.55</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>12.52</v>
+        <v>9.16</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>13.91</v>
+        <v>13.96</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14.55</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>12.6</v>
+        <v>16.75</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>12.06</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Chilaka</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>8.33</v>
+        <v>12.5</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>13.73</v>
+        <v>13.59</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>12.37</v>
+        <v>10</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>12.73</v>
+        <v>13.04</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>10.55</v>
+        <v>10.72</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>9.16</v>
+        <v>12.52</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>13.96</v>
+        <v>13.91</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.92</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>11.47</v>
+        <v>12.43</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>12.58</v>
       </c>
     </row>
     <row r="7">
@@ -1237,10 +1273,13 @@
         <v>13.93</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>14.58</v>
+      </c>
+      <c r="J7" s="6" t="n">
         <v>12.07</v>
       </c>
-      <c r="J7" s="9" t="n">
-        <v>11.63</v>
+      <c r="K7" s="9" t="n">
+        <v>11.95</v>
       </c>
     </row>
     <row r="8">
@@ -1271,10 +1310,13 @@
         <v>13.58</v>
       </c>
       <c r="I8" s="6" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="J8" s="6" t="n">
         <v>14.17</v>
       </c>
-      <c r="J8" s="9" t="n">
-        <v>11.94</v>
+      <c r="K8" s="9" t="n">
+        <v>11.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add class 2026-06-02 (part 1, 69.5 min, 10 classes total)
</commit_message>
<xml_diff>
--- a/docs/Component_A_Aggregated.xlsx
+++ b/docs/Component_A_Aggregated.xlsx
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-01 20:19 · 9 classes</t>
+          <t>Generated: 2026-06-02 15:04 · 10 classes</t>
         </is>
       </c>
     </row>
@@ -594,33 +594,33 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2.94</v>
+        <v>2.97</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="6" t="n">
-        <v>3.65</v>
+        <v>3.72</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>11.59</v>
+        <v>11.69</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>58</v>
+        <v>58.5</v>
       </c>
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="6" t="n">
-        <v>5.15</v>
+        <v>5.22</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>13.09</v>
+        <v>13.19</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>65.5</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
@@ -630,27 +630,27 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>2.97</v>
+        <v>2.93</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="6" t="n">
-        <v>3.41</v>
+        <v>3.43</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>11.39</v>
+        <v>11.36</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>57</v>
+        <v>56.8</v>
       </c>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="6" t="n">
-        <v>4.08</v>
+        <v>4.13</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>12.06</v>
@@ -666,17 +666,17 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2.44</v>
+        <v>2.42</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
       <c r="F7" s="6" t="n">
-        <v>3.86</v>
+        <v>3.88</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>11.31</v>
@@ -686,13 +686,13 @@
       </c>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="6" t="n">
-        <v>5.14</v>
+        <v>5.13</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>12.58</v>
+        <v>12.56</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>62.9</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="8">
@@ -702,33 +702,33 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="6" t="n">
-        <v>3.19</v>
+        <v>3.33</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.12</v>
+        <v>11.26</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>55.6</v>
+        <v>56.3</v>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="6" t="n">
-        <v>4.02</v>
+        <v>4.18</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>11.95</v>
+        <v>12.11</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>59.7</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="9">
@@ -738,33 +738,33 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2.32</v>
+        <v>2.4</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="6" t="n">
-        <v>3.31</v>
+        <v>3.38</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>10.63</v>
+        <v>10.78</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>53.2</v>
+        <v>53.9</v>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="6" t="n">
-        <v>4.59</v>
+        <v>4.68</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>11.91</v>
+        <v>12.08</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>59.6</v>
+        <v>60.4</v>
       </c>
     </row>
   </sheetData>
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -792,6 +792,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -852,7 +853,12 @@
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="K3" s="12" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
@@ -891,8 +897,11 @@
       <c r="J4" s="6" t="n">
         <v>11.53</v>
       </c>
-      <c r="K4" s="7" t="n">
-        <v>11.59</v>
+      <c r="K4" s="6" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>11.69</v>
       </c>
     </row>
     <row r="5">
@@ -928,8 +937,11 @@
       <c r="J5" s="6" t="n">
         <v>10.42</v>
       </c>
-      <c r="K5" s="7" t="n">
-        <v>11.39</v>
+      <c r="K5" s="6" t="n">
+        <v>11.12</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>11.36</v>
       </c>
     </row>
     <row r="6">
@@ -965,7 +977,10 @@
       <c r="J6" s="6" t="n">
         <v>13.05</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="K6" s="6" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="L6" s="7" t="n">
         <v>11.31</v>
       </c>
     </row>
@@ -1002,8 +1017,11 @@
       <c r="J7" s="6" t="n">
         <v>11.07</v>
       </c>
-      <c r="K7" s="7" t="n">
-        <v>11.12</v>
+      <c r="K7" s="6" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>11.26</v>
       </c>
     </row>
     <row r="8">
@@ -1039,8 +1057,11 @@
       <c r="J8" s="6" t="n">
         <v>12.67</v>
       </c>
-      <c r="K8" s="7" t="n">
-        <v>10.63</v>
+      <c r="K8" s="6" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>10.78</v>
       </c>
     </row>
   </sheetData>
@@ -1054,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1068,6 +1089,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1128,7 +1150,12 @@
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
@@ -1167,8 +1194,11 @@
       <c r="J4" s="6" t="n">
         <v>13.03</v>
       </c>
-      <c r="K4" s="9" t="n">
-        <v>13.09</v>
+      <c r="K4" s="6" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>13.19</v>
       </c>
     </row>
     <row r="5">
@@ -1204,7 +1234,10 @@
       <c r="J5" s="6" t="n">
         <v>10.92</v>
       </c>
-      <c r="K5" s="9" t="n">
+      <c r="K5" s="6" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="L5" s="9" t="n">
         <v>12.06</v>
       </c>
     </row>
@@ -1241,8 +1274,11 @@
       <c r="J6" s="6" t="n">
         <v>14.55</v>
       </c>
-      <c r="K6" s="9" t="n">
-        <v>12.58</v>
+      <c r="K6" s="6" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>12.56</v>
       </c>
     </row>
     <row r="7">
@@ -1278,8 +1314,11 @@
       <c r="J7" s="6" t="n">
         <v>12.07</v>
       </c>
-      <c r="K7" s="9" t="n">
-        <v>11.95</v>
+      <c r="K7" s="6" t="n">
+        <v>13.47</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>12.11</v>
       </c>
     </row>
     <row r="8">
@@ -1315,8 +1354,11 @@
       <c r="J8" s="6" t="n">
         <v>14.17</v>
       </c>
-      <c r="K8" s="9" t="n">
-        <v>11.91</v>
+      <c r="K8" s="6" t="n">
+        <v>13.61</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>12.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update 2026-06-02 with part 2 (93 min total, 948 segments)
</commit_message>
<xml_diff>
--- a/docs/Component_A_Aggregated.xlsx
+++ b/docs/Component_A_Aggregated.xlsx
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-02 15:04 · 10 classes</t>
+          <t>Generated: 2026-06-02 15:47 · 10 classes</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2.42</v>
+        <v>2.43</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>5</v>
@@ -705,30 +705,30 @@
         <v>10</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2.92</v>
+        <v>2.93</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="6" t="n">
-        <v>3.33</v>
+        <v>3.29</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.26</v>
+        <v>11.22</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>56.3</v>
+        <v>56.1</v>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="6" t="n">
-        <v>4.18</v>
+        <v>4.19</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>12.11</v>
+        <v>12.12</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>60.5</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="9">
@@ -741,30 +741,30 @@
         <v>10</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="6" t="n">
-        <v>3.38</v>
+        <v>3.36</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>10.78</v>
+        <v>10.75</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>53.9</v>
+        <v>53.8</v>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="6" t="n">
-        <v>4.68</v>
+        <v>4.66</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>12.08</v>
+        <v>12.05</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>60.4</v>
+        <v>60.2</v>
       </c>
     </row>
   </sheetData>
@@ -898,7 +898,7 @@
         <v>11.53</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>12.55</v>
+        <v>12.58</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>11.69</v>
@@ -978,7 +978,7 @@
         <v>13.05</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>11.3</v>
+        <v>11.32</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>11.31</v>
@@ -1018,10 +1018,10 @@
         <v>11.07</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>12.47</v>
+        <v>12.1</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>11.26</v>
+        <v>11.22</v>
       </c>
     </row>
     <row r="8">
@@ -1058,10 +1058,10 @@
         <v>12.67</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>12.11</v>
+        <v>11.82</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>10.78</v>
+        <v>10.75</v>
       </c>
     </row>
   </sheetData>
@@ -1195,7 +1195,7 @@
         <v>13.03</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>14.05</v>
+        <v>14.08</v>
       </c>
       <c r="L4" s="9" t="n">
         <v>13.19</v>
@@ -1275,7 +1275,7 @@
         <v>14.55</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>12.3</v>
+        <v>12.32</v>
       </c>
       <c r="L6" s="9" t="n">
         <v>12.56</v>
@@ -1315,10 +1315,10 @@
         <v>12.07</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>13.47</v>
+        <v>13.6</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>12.11</v>
+        <v>12.12</v>
       </c>
     </row>
     <row r="8">
@@ -1355,10 +1355,10 @@
         <v>14.17</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>13.61</v>
+        <v>13.32</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>12.08</v>
+        <v>12.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update 2026-06-02 with part 3 (133 min total, 1134 segments)
</commit_message>
<xml_diff>
--- a/docs/Component_A_Aggregated.xlsx
+++ b/docs/Component_A_Aggregated.xlsx
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-02 15:47 · 10 classes</t>
+          <t>Generated: 2026-06-02 16:18 · 10 classes</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2.97</v>
+        <v>2.98</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>5</v>
@@ -686,13 +686,13 @@
       </c>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="6" t="n">
-        <v>5.13</v>
+        <v>5.18</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>12.56</v>
+        <v>12.61</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>62.8</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8">
@@ -705,7 +705,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>5</v>
@@ -715,20 +715,20 @@
         <v>3.29</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.22</v>
+        <v>11.2</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>56.1</v>
+        <v>56</v>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="6" t="n">
         <v>4.19</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>12.12</v>
+        <v>12.1</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>60.6</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="9">
@@ -751,7 +751,7 @@
         <v>3.36</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>10.75</v>
+        <v>10.76</v>
       </c>
       <c r="H9" s="8" t="n">
         <v>53.8</v>
@@ -761,10 +761,10 @@
         <v>4.66</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>12.05</v>
+        <v>12.06</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
     </row>
   </sheetData>
@@ -898,7 +898,7 @@
         <v>11.53</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>12.58</v>
+        <v>12.61</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>11.69</v>
@@ -938,7 +938,7 @@
         <v>10.42</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>11.12</v>
+        <v>11.08</v>
       </c>
       <c r="L5" s="7" t="n">
         <v>11.36</v>
@@ -978,7 +978,7 @@
         <v>13.05</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>11.32</v>
+        <v>11.34</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>11.31</v>
@@ -1018,10 +1018,10 @@
         <v>11.07</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>12.1</v>
+        <v>11.93</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>11.22</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="8">
@@ -1058,10 +1058,10 @@
         <v>12.67</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>11.82</v>
+        <v>11.9</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>10.75</v>
+        <v>10.76</v>
       </c>
     </row>
   </sheetData>
@@ -1195,7 +1195,7 @@
         <v>13.03</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>14.08</v>
+        <v>14.11</v>
       </c>
       <c r="L4" s="9" t="n">
         <v>13.19</v>
@@ -1235,7 +1235,7 @@
         <v>10.92</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>12.12</v>
+        <v>12.08</v>
       </c>
       <c r="L5" s="9" t="n">
         <v>12.06</v>
@@ -1275,10 +1275,10 @@
         <v>14.55</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>12.32</v>
+        <v>12.84</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>12.56</v>
+        <v>12.61</v>
       </c>
     </row>
     <row r="7">
@@ -1315,10 +1315,10 @@
         <v>12.07</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>13.6</v>
+        <v>13.43</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>12.12</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="8">
@@ -1355,10 +1355,10 @@
         <v>14.17</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>13.32</v>
+        <v>13.4</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>12.05</v>
+        <v>12.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>